<commit_message>
current state monday am 23rd feb
</commit_message>
<xml_diff>
--- a/data/raw/2025/natcan6_070925.xlsx
+++ b/data/raw/2025/natcan6_070925.xlsx
@@ -18,7 +18,7 @@
     <sheet name="perpPara_090925" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -688,6 +688,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>